<commit_message>
Add EBA SOT, enhanced ALM report, and IRRBB/LCR improvements
- Add EBA IRRBB Supervisory Outlier Test (eba_sot_objects.py, eba_sot_workflow.py)
- Add bank_report.ipynb with full ALM dashboard: balance sheet product detail,
  IRS book profile, NM vs term deposit run-off split, outstanding notionals,
  rate sensitivity heatmap, repricing ladder, NII/EVE tornado charts
- Fix IR gap legend (green/red patches + IRS clarification in titles)
- Extend nii/eve calc objects and workflows with rate limits, shocked CF tables
- Add LCR/NSFR workflow enhancements and updated output reports
- Update balance sheet and IRS input data

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/balance_generate/input_data/bank_data.xlsx
+++ b/balance_generate/input_data/bank_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dzimi\Documents\data_engineering\data_projects\git_hub_projects\bank_project\balance_generate\input_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C55AD9B5-26E6-4E41-9D01-A9508F3687D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C9E8C0C-997F-4B5E-B1E8-D77343F261AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3640" yWindow="3640" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="bs_structure" sheetId="2" r:id="rId1"/>
@@ -697,7 +697,7 @@
         <v>45657</v>
       </c>
       <c r="B2">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C2" t="s">
         <v>0</v>
@@ -930,7 +930,7 @@
         <v>45657</v>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C6" t="s">
         <v>0</v>
@@ -1051,7 +1051,7 @@
         <v>45657</v>
       </c>
       <c r="B8">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C8" t="s">
         <v>0</v>
@@ -1181,7 +1181,7 @@
         <v>45657</v>
       </c>
       <c r="B10">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="C10" t="s">
         <v>0</v>
@@ -1231,8 +1231,8 @@
       <c r="R10" t="s">
         <v>32</v>
       </c>
-      <c r="W10">
-        <v>1</v>
+      <c r="X10">
+        <v>0.8</v>
       </c>
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.35">
@@ -1240,7 +1240,7 @@
         <v>45657</v>
       </c>
       <c r="B11">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C11" t="s">
         <v>1</v>
@@ -1529,7 +1529,7 @@
         <v>45657</v>
       </c>
       <c r="B16">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C16" t="s">
         <v>1</v>
@@ -1673,7 +1673,7 @@
         <v>45657</v>
       </c>
       <c r="B19">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C19" t="s">
         <v>2</v>

</xml_diff>

<commit_message>
Update LabBank Streamlit sandbox app and its data dependencies
Scoped to what sandbox/app.py's import graph actually reads: the app
code itself plus the six data files it loads directly (scenario
curves cache, product/curve tensors, bank_data.xlsx, irs_input.xlsx,
dep_beh_models_ir.xlsx) -- needed so a Streamlit Community Cloud
deploy pointed at sandbox/app.py has current data to read.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/balance_generate/input_data/bank_data.xlsx
+++ b/balance_generate/input_data/bank_data.xlsx
@@ -1111,7 +1111,7 @@
         <v>45657</v>
       </c>
       <c r="B7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1217,7 +1217,7 @@
         <v>45657</v>
       </c>
       <c r="B8" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -2393,7 +2393,7 @@
         <v>45657</v>
       </c>
       <c r="B20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>

</xml_diff>